<commit_message>
Inclui o Relatório CFTV de 06/10/2026 com câmeras reconciliadas pelo histórico
- período 01/09–06/10; 25/09–05/10 sem arquivo (colunas brancas, nada inventado)
- nova regra (decisão da Letícia em 07/10/2026, REGRAS §17-A): a partir de 06/10, quando as câmeras
  do relatório não batem com o registro anterior do veículo e a quantidade é a mesma, os valores
  passam para os números do histórico (troca de coluna, sem criar/apagar valores); quantidade
  diferente fica como veio e é listada na Auditoria
- 06/10: 463 veículos remapeados (ALFA RODOBUS 142, ALFA RODOBUS SPE 123, NORTE BUSS A2 198)
  e 91 mantidos (quantidade de câmeras diferente do histórico)
- resultados: RESOLVIDO 79, COM RECORRÊNCIA 27, NÃO RESOLVIDO 50, PARCIAL 18, SEM DADOS 139;
  taxa de resolução 79 ÷ 174 = 45,4%
- textos do período/Auditoria sem datas fixas; teste da reconciliação; testar_publicado com os
  novos números e checagem da coluna 06/10
</commit_message>
<xml_diff>
--- a/data/processed/manutencao_x_cftv.xlsx
+++ b/data/processed/manutencao_x_cftv.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3514" uniqueCount="1046">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3561" uniqueCount="1070">
   <si>
     <t>evento</t>
   </si>
@@ -2929,229 +2929,301 @@
     <t>CORREDOR 1 (câm 23) ONLINE COM ERRO (SD: error, Gravação: error); CORREDOR 2 (câm 24) ONLINE COM ERRO (SD: error, Gravação: error); CORREDOR 4 (câm 26) OFFLINE</t>
   </si>
   <si>
-    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-15 VERMELHO | 2026-09-16 VERMELHO | 2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
+    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-15 VERMELHO | 2026-09-16 VERMELHO | 2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
   </si>
   <si>
     <t>2026-09-15 VERMELHO | 2026-09-16 VERMELHO | 2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO</t>
   </si>
   <si>
-    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-15 VERDE | 2026-09-16 LARANJA | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-15 LARANJA | 2026-09-16 LARANJA | 2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
+    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-15 VERDE | 2026-09-16 LARANJA | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-24 LARANJA | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-15 LARANJA | 2026-09-16 LARANJA | 2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-15 VERMELHO | 2026-09-16 VERMELHO | 2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERDE</t>
   </si>
   <si>
     <t>2026-09-15 VERDE | 2026-09-16 VERDE</t>
   </si>
   <si>
-    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-15 LARANJA | 2026-09-16 LARANJA | 2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
+    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-15 LARANJA | 2026-09-16 LARANJA | 2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
   </si>
   <si>
     <t>2026-09-15 LARANJA</t>
   </si>
   <si>
-    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-16 LARANJA | 2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-16 VERMELHO | 2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
+    <t>2026-09-15 VERDE | 2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-16 LARANJA | 2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-16 VERMELHO | 2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
   </si>
   <si>
     <t>2026-09-16 LARANJA | 2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA</t>
   </si>
   <si>
-    <t>2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
+    <t>2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
   </si>
   <si>
     <t>2026-09-16 LARANJA | 2026-09-17 LARANJA | 2026-09-18 LARANJA</t>
   </si>
   <si>
+    <t>2026-09-16 LARANJA | 2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
     <t>2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE</t>
   </si>
   <si>
-    <t>2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 VERMELHO | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERMELHO | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERMELHO | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-17 LARANJA | 2026-09-18 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-17 LARANJA | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 LARANJA | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
+    <t>2026-09-16 VERDE | 2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 VERMELHO | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERMELHO | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERMELHO | 2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-17 LARANJA | 2026-09-18 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-17 LARANJA | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 LARANJA | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-17 LARANJA | 2026-09-18 LARANJA | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
   </si>
   <si>
     <t>2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-21 VERMELHO</t>
   </si>
   <si>
-    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERMELHO | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERDE | 2026-09-21 VERDE | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERMELHO | 2026-09-18 LARANJA | 2026-09-21 VERMELHO | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-18 VERDE | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERMELHO | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERMELHO | 2026-09-18 VERMELHO | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-21 VERDE | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERMELHO | 2026-09-18 LARANJA | 2026-09-21 VERMELHO | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 VERMELHO | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-17 VERDE | 2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-18 VERDE | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
   </si>
   <si>
     <t>2026-09-18 VERDE</t>
   </si>
   <si>
-    <t>2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-18 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 VERDE | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-18 VERDE | 2026-09-21 VERMELHO | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
+    <t>2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-18 VERMELHO | 2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-18 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 VERDE | 2026-09-24 LARANJA | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-18 VERDE | 2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-18 VERDE | 2026-09-21 VERMELHO | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-18 LARANJA | 2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERDE</t>
   </si>
   <si>
     <t>2026-09-21 LARANJA | 2026-09-22 VERMELHO | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
   </si>
   <si>
-    <t>2026-09-21 LARANJA | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERMELHO | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-21 VERMELHO | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-22 VERMELHO | 2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-22 VERMELHO | 2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-23 VERDE | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-23 VERMELHO | 2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-23 LARANJA | 2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-23 VERMELHO | 2026-09-24 VERMELHO</t>
-  </si>
-  <si>
-    <t>2026-09-24 VERDE</t>
-  </si>
-  <si>
-    <t>2026-09-24 LARANJA</t>
-  </si>
-  <si>
-    <t>2026-09-24 VERMELHO</t>
+    <t>2026-09-21 LARANJA | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-21 LARANJA | 2026-09-22 LARANJA | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERMELHO | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-21 VERMELHO | 2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-21 LARANJA | 2026-09-22 VERMELHO | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-21 VERDE | 2026-09-22 VERDE | 2026-09-23 VERMELHO | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-21 VERMELHO | 2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-22 VERMELHO | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-22 VERDE | 2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-22 VERMELHO | 2026-09-23 VERMELHO | 2026-09-24 VERDE | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-22 VERMELHO | 2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-23 VERDE | 2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-23 VERMELHO | 2026-09-24 VERDE | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-23 LARANJA | 2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-23 VERMELHO | 2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-24 VERDE | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-09-24 LARANJA | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-24 VERDE | 2026-10-06 LARANJA</t>
+  </si>
+  <si>
+    <t>2026-09-24 LARANJA | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-24 VERMELHO | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-24 VERDE | 2026-10-06 VERMELHO</t>
+  </si>
+  <si>
+    <t>2026-09-24 VERMELHO | 2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-10-06 VERDE</t>
+  </si>
+  <si>
+    <t>2026-10-06 LARANJA</t>
   </si>
 </sst>
 </file>
@@ -3571,7 +3643,7 @@
         <v>922</v>
       </c>
       <c r="M2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N2" t="s">
         <v>971</v>
@@ -3615,7 +3687,7 @@
         <v>921</v>
       </c>
       <c r="M3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N3" t="s">
         <v>972</v>
@@ -3659,7 +3731,7 @@
         <v>921</v>
       </c>
       <c r="M4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N4" t="s">
         <v>972</v>
@@ -3703,7 +3775,7 @@
         <v>921</v>
       </c>
       <c r="M5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N5" t="s">
         <v>972</v>
@@ -3791,7 +3863,7 @@
         <v>921</v>
       </c>
       <c r="M7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N7" t="s">
         <v>972</v>
@@ -3832,7 +3904,7 @@
         <v>922</v>
       </c>
       <c r="M8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N8" t="s">
         <v>974</v>
@@ -3873,7 +3945,7 @@
         <v>922</v>
       </c>
       <c r="M9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N9" t="s">
         <v>975</v>
@@ -3917,7 +3989,7 @@
         <v>920</v>
       </c>
       <c r="M10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N10" t="s">
         <v>974</v>
@@ -3961,7 +4033,7 @@
         <v>921</v>
       </c>
       <c r="M11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N11" t="s">
         <v>976</v>
@@ -3999,7 +4071,7 @@
         <v>922</v>
       </c>
       <c r="M12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N12" t="s">
         <v>974</v>
@@ -4040,7 +4112,7 @@
         <v>931</v>
       </c>
       <c r="M13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N13" t="s">
         <v>977</v>
@@ -4081,7 +4153,7 @@
         <v>932</v>
       </c>
       <c r="M14">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N14" t="s">
         <v>978</v>
@@ -4122,10 +4194,10 @@
         <v>930</v>
       </c>
       <c r="M15">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N15" t="s">
-        <v>972</v>
+        <v>979</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -4160,7 +4232,7 @@
         <v>922</v>
       </c>
       <c r="M16">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N16" t="s">
         <v>974</v>
@@ -4201,7 +4273,7 @@
         <v>2</v>
       </c>
       <c r="N17" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="O17" t="s">
         <v>333</v>
@@ -4239,7 +4311,7 @@
         <v>922</v>
       </c>
       <c r="M18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N18" t="s">
         <v>974</v>
@@ -4280,7 +4352,7 @@
         <v>933</v>
       </c>
       <c r="M19">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N19" t="s">
         <v>972</v>
@@ -4318,10 +4390,10 @@
         <v>922</v>
       </c>
       <c r="M20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N20" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
     </row>
     <row r="21" spans="1:15">
@@ -4359,7 +4431,7 @@
         <v>930</v>
       </c>
       <c r="M21">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N21" t="s">
         <v>974</v>
@@ -4400,10 +4472,10 @@
         <v>932</v>
       </c>
       <c r="M22">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N22" t="s">
-        <v>974</v>
+        <v>982</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -4441,10 +4513,10 @@
         <v>934</v>
       </c>
       <c r="M23">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N23" t="s">
-        <v>981</v>
+        <v>983</v>
       </c>
     </row>
     <row r="24" spans="1:15">
@@ -4482,10 +4554,10 @@
         <v>929</v>
       </c>
       <c r="M24">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N24" t="s">
-        <v>982</v>
+        <v>984</v>
       </c>
     </row>
     <row r="25" spans="1:15">
@@ -4523,7 +4595,7 @@
         <v>935</v>
       </c>
       <c r="M25">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N25" t="s">
         <v>978</v>
@@ -4564,10 +4636,10 @@
         <v>927</v>
       </c>
       <c r="M26">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N26" t="s">
-        <v>983</v>
+        <v>985</v>
       </c>
     </row>
     <row r="27" spans="1:15">
@@ -4608,7 +4680,7 @@
         <v>1</v>
       </c>
       <c r="N27" t="s">
-        <v>984</v>
+        <v>986</v>
       </c>
       <c r="O27" t="s">
         <v>332</v>
@@ -4649,7 +4721,7 @@
         <v>927</v>
       </c>
       <c r="M28">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N28" t="s">
         <v>974</v>
@@ -4690,7 +4762,7 @@
         <v>936</v>
       </c>
       <c r="M29">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N29" t="s">
         <v>978</v>
@@ -4728,10 +4800,10 @@
         <v>922</v>
       </c>
       <c r="M30">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N30" t="s">
-        <v>985</v>
+        <v>987</v>
       </c>
     </row>
     <row r="31" spans="1:15">
@@ -4769,10 +4841,10 @@
         <v>922</v>
       </c>
       <c r="M31">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N31" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="32" spans="1:15">
@@ -4810,10 +4882,10 @@
         <v>922</v>
       </c>
       <c r="M32">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N32" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="33" spans="1:15">
@@ -4851,10 +4923,10 @@
         <v>922</v>
       </c>
       <c r="M33">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N33" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
     </row>
     <row r="34" spans="1:15">
@@ -4892,10 +4964,10 @@
         <v>922</v>
       </c>
       <c r="M34">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N34" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="35" spans="1:15">
@@ -4933,10 +5005,10 @@
         <v>922</v>
       </c>
       <c r="M35">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N35" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="36" spans="1:15">
@@ -4974,10 +5046,10 @@
         <v>922</v>
       </c>
       <c r="M36">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N36" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="37" spans="1:15">
@@ -5015,10 +5087,10 @@
         <v>922</v>
       </c>
       <c r="M37">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N37" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="38" spans="1:15">
@@ -5059,10 +5131,10 @@
         <v>920</v>
       </c>
       <c r="M38">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N38" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
     </row>
     <row r="39" spans="1:15">
@@ -5103,10 +5175,10 @@
         <v>920</v>
       </c>
       <c r="M39">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N39" t="s">
-        <v>988</v>
+        <v>991</v>
       </c>
     </row>
     <row r="40" spans="1:15">
@@ -5147,10 +5219,10 @@
         <v>921</v>
       </c>
       <c r="M40">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N40" t="s">
-        <v>989</v>
+        <v>992</v>
       </c>
     </row>
     <row r="41" spans="1:15">
@@ -5191,10 +5263,10 @@
         <v>922</v>
       </c>
       <c r="M41">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N41" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="42" spans="1:15">
@@ -5232,10 +5304,10 @@
         <v>922</v>
       </c>
       <c r="M42">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N42" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="43" spans="1:15">
@@ -5276,10 +5348,10 @@
         <v>921</v>
       </c>
       <c r="M43">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N43" t="s">
-        <v>989</v>
+        <v>992</v>
       </c>
     </row>
     <row r="44" spans="1:15">
@@ -5320,7 +5392,7 @@
         <v>5</v>
       </c>
       <c r="N44" t="s">
-        <v>990</v>
+        <v>993</v>
       </c>
       <c r="O44" t="s">
         <v>339</v>
@@ -5408,10 +5480,10 @@
         <v>922</v>
       </c>
       <c r="M46">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N46" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="47" spans="1:15">
@@ -5449,10 +5521,10 @@
         <v>922</v>
       </c>
       <c r="M47">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N47" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="48" spans="1:15">
@@ -5493,10 +5565,10 @@
         <v>922</v>
       </c>
       <c r="M48">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N48" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="49" spans="1:15">
@@ -5537,10 +5609,10 @@
         <v>922</v>
       </c>
       <c r="M49">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N49" t="s">
-        <v>991</v>
+        <v>994</v>
       </c>
     </row>
     <row r="50" spans="1:15">
@@ -5584,7 +5656,7 @@
         <v>3</v>
       </c>
       <c r="N50" t="s">
-        <v>992</v>
+        <v>995</v>
       </c>
       <c r="O50" t="s">
         <v>335</v>
@@ -5625,10 +5697,10 @@
         <v>922</v>
       </c>
       <c r="M51">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N51" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="52" spans="1:15">
@@ -5669,10 +5741,10 @@
         <v>920</v>
       </c>
       <c r="M52">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N52" t="s">
-        <v>987</v>
+        <v>996</v>
       </c>
     </row>
     <row r="53" spans="1:15">
@@ -5713,7 +5785,7 @@
         <v>4</v>
       </c>
       <c r="N53" t="s">
-        <v>993</v>
+        <v>997</v>
       </c>
     </row>
     <row r="54" spans="1:15">
@@ -5751,10 +5823,10 @@
         <v>922</v>
       </c>
       <c r="M54">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N54" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="55" spans="1:15">
@@ -5833,10 +5905,10 @@
         <v>922</v>
       </c>
       <c r="M56">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N56" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="57" spans="1:15">
@@ -5877,10 +5949,10 @@
         <v>920</v>
       </c>
       <c r="M57">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N57" t="s">
-        <v>987</v>
+        <v>996</v>
       </c>
     </row>
     <row r="58" spans="1:15">
@@ -5918,10 +5990,10 @@
         <v>922</v>
       </c>
       <c r="M58">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N58" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="59" spans="1:15">
@@ -5962,10 +6034,10 @@
         <v>920</v>
       </c>
       <c r="M59">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N59" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
     </row>
     <row r="60" spans="1:15">
@@ -6006,10 +6078,10 @@
         <v>921</v>
       </c>
       <c r="M60">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N60" t="s">
-        <v>989</v>
+        <v>992</v>
       </c>
     </row>
     <row r="61" spans="1:15">
@@ -6050,10 +6122,10 @@
         <v>921</v>
       </c>
       <c r="M61">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N61" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
     </row>
     <row r="62" spans="1:15">
@@ -6094,10 +6166,10 @@
         <v>922</v>
       </c>
       <c r="M62">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N62" t="s">
-        <v>986</v>
+        <v>998</v>
       </c>
     </row>
     <row r="63" spans="1:15">
@@ -6138,10 +6210,10 @@
         <v>920</v>
       </c>
       <c r="M63">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N63" t="s">
-        <v>994</v>
+        <v>999</v>
       </c>
     </row>
     <row r="64" spans="1:15">
@@ -6182,10 +6254,10 @@
         <v>920</v>
       </c>
       <c r="M64">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N64" t="s">
-        <v>995</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="65" spans="1:14">
@@ -6226,10 +6298,10 @@
         <v>920</v>
       </c>
       <c r="M65">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N65" t="s">
-        <v>995</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="66" spans="1:14">
@@ -6267,10 +6339,10 @@
         <v>922</v>
       </c>
       <c r="M66">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N66" t="s">
-        <v>996</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="67" spans="1:14">
@@ -6311,10 +6383,10 @@
         <v>920</v>
       </c>
       <c r="M67">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N67" t="s">
-        <v>997</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="68" spans="1:14">
@@ -6355,10 +6427,10 @@
         <v>921</v>
       </c>
       <c r="M68">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N68" t="s">
-        <v>998</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="69" spans="1:14">
@@ -6399,10 +6471,10 @@
         <v>920</v>
       </c>
       <c r="M69">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N69" t="s">
-        <v>995</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="70" spans="1:14">
@@ -6443,10 +6515,10 @@
         <v>922</v>
       </c>
       <c r="M70">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N70" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="71" spans="1:14">
@@ -6484,10 +6556,10 @@
         <v>922</v>
       </c>
       <c r="M71">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N71" t="s">
-        <v>996</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="72" spans="1:14">
@@ -6525,10 +6597,10 @@
         <v>922</v>
       </c>
       <c r="M72">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N72" t="s">
-        <v>999</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="73" spans="1:14">
@@ -6566,10 +6638,10 @@
         <v>922</v>
       </c>
       <c r="M73">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N73" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="74" spans="1:14">
@@ -6610,10 +6682,10 @@
         <v>922</v>
       </c>
       <c r="M74">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N74" t="s">
-        <v>996</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="75" spans="1:14">
@@ -6651,10 +6723,10 @@
         <v>922</v>
       </c>
       <c r="M75">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N75" t="s">
-        <v>1000</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="76" spans="1:14">
@@ -6692,10 +6764,10 @@
         <v>922</v>
       </c>
       <c r="M76">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N76" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="77" spans="1:14">
@@ -6736,10 +6808,10 @@
         <v>921</v>
       </c>
       <c r="M77">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N77" t="s">
-        <v>998</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="78" spans="1:14">
@@ -6777,10 +6849,10 @@
         <v>922</v>
       </c>
       <c r="M78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N78" t="s">
-        <v>1001</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="79" spans="1:14">
@@ -6821,10 +6893,10 @@
         <v>922</v>
       </c>
       <c r="M79">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N79" t="s">
-        <v>996</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="80" spans="1:14">
@@ -6865,10 +6937,10 @@
         <v>922</v>
       </c>
       <c r="M80">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N80" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="81" spans="1:14">
@@ -6909,10 +6981,10 @@
         <v>921</v>
       </c>
       <c r="M81">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N81" t="s">
-        <v>998</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="82" spans="1:14">
@@ -6953,10 +7025,10 @@
         <v>922</v>
       </c>
       <c r="M82">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N82" t="s">
-        <v>1002</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="83" spans="1:14">
@@ -6997,10 +7069,10 @@
         <v>922</v>
       </c>
       <c r="M83">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N83" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="84" spans="1:14">
@@ -7041,10 +7113,10 @@
         <v>922</v>
       </c>
       <c r="M84">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N84" t="s">
-        <v>996</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="85" spans="1:14">
@@ -7085,10 +7157,10 @@
         <v>922</v>
       </c>
       <c r="M85">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N85" t="s">
-        <v>1000</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="86" spans="1:14">
@@ -7129,10 +7201,10 @@
         <v>922</v>
       </c>
       <c r="M86">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N86" t="s">
-        <v>998</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="87" spans="1:14">
@@ -7173,10 +7245,10 @@
         <v>922</v>
       </c>
       <c r="M87">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N87" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="88" spans="1:14">
@@ -7217,10 +7289,10 @@
         <v>922</v>
       </c>
       <c r="M88">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N88" t="s">
-        <v>1000</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="89" spans="1:14">
@@ -7261,10 +7333,10 @@
         <v>922</v>
       </c>
       <c r="M89">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N89" t="s">
-        <v>1003</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="90" spans="1:14">
@@ -7305,10 +7377,10 @@
         <v>922</v>
       </c>
       <c r="M90">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N90" t="s">
-        <v>995</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="91" spans="1:14">
@@ -7346,10 +7418,10 @@
         <v>922</v>
       </c>
       <c r="M91">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N91" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="92" spans="1:14">
@@ -7387,10 +7459,10 @@
         <v>922</v>
       </c>
       <c r="M92">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N92" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="93" spans="1:14">
@@ -7431,10 +7503,10 @@
         <v>922</v>
       </c>
       <c r="M93">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N93" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="94" spans="1:14">
@@ -7475,10 +7547,10 @@
         <v>922</v>
       </c>
       <c r="M94">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N94" t="s">
-        <v>1004</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="95" spans="1:14">
@@ -7519,10 +7591,10 @@
         <v>922</v>
       </c>
       <c r="M95">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N95" t="s">
-        <v>1005</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="96" spans="1:14">
@@ -7563,10 +7635,10 @@
         <v>921</v>
       </c>
       <c r="M96">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N96" t="s">
-        <v>998</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="97" spans="1:14">
@@ -7607,10 +7679,10 @@
         <v>922</v>
       </c>
       <c r="M97">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N97" t="s">
-        <v>1006</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="98" spans="1:14">
@@ -7651,10 +7723,10 @@
         <v>922</v>
       </c>
       <c r="M98">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N98" t="s">
-        <v>1007</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="99" spans="1:14">
@@ -7695,10 +7767,10 @@
         <v>922</v>
       </c>
       <c r="M99">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N99" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="100" spans="1:14">
@@ -7739,10 +7811,10 @@
         <v>922</v>
       </c>
       <c r="M100">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N100" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="101" spans="1:14">
@@ -7783,10 +7855,10 @@
         <v>920</v>
       </c>
       <c r="M101">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N101" t="s">
-        <v>1008</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="102" spans="1:14">
@@ -7824,10 +7896,10 @@
         <v>922</v>
       </c>
       <c r="M102">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N102" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="103" spans="1:14">
@@ -7865,10 +7937,10 @@
         <v>922</v>
       </c>
       <c r="M103">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N103" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="104" spans="1:14">
@@ -7906,10 +7978,10 @@
         <v>922</v>
       </c>
       <c r="M104">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N104" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="105" spans="1:14">
@@ -7953,7 +8025,7 @@
         <v>3</v>
       </c>
       <c r="N105" t="s">
-        <v>1009</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="106" spans="1:14">
@@ -7997,7 +8069,7 @@
         <v>3</v>
       </c>
       <c r="N106" t="s">
-        <v>1009</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="107" spans="1:14">
@@ -8035,10 +8107,10 @@
         <v>922</v>
       </c>
       <c r="M107">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N107" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="108" spans="1:14">
@@ -8076,10 +8148,10 @@
         <v>922</v>
       </c>
       <c r="M108">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N108" t="s">
-        <v>1010</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="109" spans="1:14">
@@ -8120,10 +8192,10 @@
         <v>921</v>
       </c>
       <c r="M109">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N109" t="s">
-        <v>998</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="110" spans="1:14">
@@ -8164,10 +8236,10 @@
         <v>922</v>
       </c>
       <c r="M110">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N110" t="s">
-        <v>996</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="111" spans="1:14">
@@ -8208,10 +8280,10 @@
         <v>920</v>
       </c>
       <c r="M111">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N111" t="s">
-        <v>1008</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="112" spans="1:14">
@@ -8249,10 +8321,10 @@
         <v>922</v>
       </c>
       <c r="M112">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N112" t="s">
-        <v>1011</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="113" spans="1:15">
@@ -8293,10 +8365,10 @@
         <v>921</v>
       </c>
       <c r="M113">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N113" t="s">
-        <v>1012</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="114" spans="1:15">
@@ -8337,10 +8409,10 @@
         <v>922</v>
       </c>
       <c r="M114">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N114" t="s">
-        <v>1013</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="115" spans="1:15">
@@ -8381,10 +8453,10 @@
         <v>920</v>
       </c>
       <c r="M115">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N115" t="s">
-        <v>1014</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="116" spans="1:15">
@@ -8425,10 +8497,10 @@
         <v>922</v>
       </c>
       <c r="M116">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N116" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="117" spans="1:15">
@@ -8466,10 +8538,10 @@
         <v>922</v>
       </c>
       <c r="M117">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N117" t="s">
-        <v>1003</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="118" spans="1:15">
@@ -8507,10 +8579,10 @@
         <v>922</v>
       </c>
       <c r="M118">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N118" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="119" spans="1:15">
@@ -8539,10 +8611,10 @@
         <v>917</v>
       </c>
       <c r="M119">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N119" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="120" spans="1:15">
@@ -8571,10 +8643,10 @@
         <v>917</v>
       </c>
       <c r="M120">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N120" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="121" spans="1:15">
@@ -8615,10 +8687,10 @@
         <v>922</v>
       </c>
       <c r="M121">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N121" t="s">
-        <v>1016</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="122" spans="1:15">
@@ -8659,10 +8731,10 @@
         <v>922</v>
       </c>
       <c r="M122">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N122" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="123" spans="1:15">
@@ -8703,10 +8775,10 @@
         <v>922</v>
       </c>
       <c r="M123">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N123" t="s">
-        <v>996</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="124" spans="1:15">
@@ -8744,10 +8816,10 @@
         <v>922</v>
       </c>
       <c r="M124">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N124" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="125" spans="1:15">
@@ -8788,10 +8860,10 @@
         <v>920</v>
       </c>
       <c r="M125">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N125" t="s">
-        <v>1018</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="126" spans="1:15">
@@ -8829,10 +8901,10 @@
         <v>922</v>
       </c>
       <c r="M126">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N126" t="s">
-        <v>1019</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="127" spans="1:15">
@@ -8870,10 +8942,10 @@
         <v>922</v>
       </c>
       <c r="M127">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N127" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="128" spans="1:15">
@@ -8917,7 +8989,7 @@
         <v>1</v>
       </c>
       <c r="N128" t="s">
-        <v>1020</v>
+        <v>1028</v>
       </c>
       <c r="O128" t="s">
         <v>335</v>
@@ -8958,10 +9030,10 @@
         <v>922</v>
       </c>
       <c r="M129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N129" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="130" spans="1:14">
@@ -8999,10 +9071,10 @@
         <v>922</v>
       </c>
       <c r="M130">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N130" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="131" spans="1:14">
@@ -9040,10 +9112,10 @@
         <v>922</v>
       </c>
       <c r="M131">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N131" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="132" spans="1:14">
@@ -9081,10 +9153,10 @@
         <v>922</v>
       </c>
       <c r="M132">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N132" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="133" spans="1:14">
@@ -9125,10 +9197,10 @@
         <v>922</v>
       </c>
       <c r="M133">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N133" t="s">
-        <v>1021</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="134" spans="1:14">
@@ -9166,10 +9238,10 @@
         <v>922</v>
       </c>
       <c r="M134">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N134" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="135" spans="1:14">
@@ -9207,10 +9279,10 @@
         <v>922</v>
       </c>
       <c r="M135">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N135" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="136" spans="1:14">
@@ -9251,10 +9323,10 @@
         <v>921</v>
       </c>
       <c r="M136">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N136" t="s">
-        <v>1022</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="137" spans="1:14">
@@ -9295,10 +9367,10 @@
         <v>920</v>
       </c>
       <c r="M137">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N137" t="s">
-        <v>1018</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="138" spans="1:14">
@@ -9339,10 +9411,10 @@
         <v>921</v>
       </c>
       <c r="M138">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N138" t="s">
-        <v>1022</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="139" spans="1:14">
@@ -9383,10 +9455,10 @@
         <v>922</v>
       </c>
       <c r="M139">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N139" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="140" spans="1:14">
@@ -9424,10 +9496,10 @@
         <v>922</v>
       </c>
       <c r="M140">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N140" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="141" spans="1:14">
@@ -9465,10 +9537,10 @@
         <v>922</v>
       </c>
       <c r="M141">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N141" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="142" spans="1:14">
@@ -9506,10 +9578,10 @@
         <v>922</v>
       </c>
       <c r="M142">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N142" t="s">
-        <v>1023</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="143" spans="1:14">
@@ -9547,10 +9619,10 @@
         <v>922</v>
       </c>
       <c r="M143">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N143" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="144" spans="1:14">
@@ -9591,10 +9663,10 @@
         <v>922</v>
       </c>
       <c r="M144">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N144" t="s">
-        <v>1024</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="145" spans="1:14">
@@ -9635,10 +9707,10 @@
         <v>922</v>
       </c>
       <c r="M145">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N145" t="s">
-        <v>1017</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="146" spans="1:14">
@@ -9679,10 +9751,10 @@
         <v>922</v>
       </c>
       <c r="M146">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N146" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="147" spans="1:14">
@@ -9720,10 +9792,10 @@
         <v>922</v>
       </c>
       <c r="M147">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N147" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="148" spans="1:14">
@@ -9761,10 +9833,10 @@
         <v>922</v>
       </c>
       <c r="M148">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N148" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="149" spans="1:14">
@@ -9802,10 +9874,10 @@
         <v>922</v>
       </c>
       <c r="M149">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N149" t="s">
-        <v>1025</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="150" spans="1:14">
@@ -9846,10 +9918,10 @@
         <v>920</v>
       </c>
       <c r="M150">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N150" t="s">
-        <v>1018</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="151" spans="1:14">
@@ -9890,10 +9962,10 @@
         <v>920</v>
       </c>
       <c r="M151">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N151" t="s">
-        <v>1018</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="152" spans="1:14">
@@ -9931,10 +10003,10 @@
         <v>922</v>
       </c>
       <c r="M152">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N152" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="153" spans="1:14">
@@ -9972,10 +10044,10 @@
         <v>922</v>
       </c>
       <c r="M153">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N153" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="154" spans="1:14">
@@ -10016,10 +10088,10 @@
         <v>920</v>
       </c>
       <c r="M154">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N154" t="s">
-        <v>1018</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="155" spans="1:14">
@@ -10060,10 +10132,10 @@
         <v>920</v>
       </c>
       <c r="M155">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N155" t="s">
-        <v>1018</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="156" spans="1:14">
@@ -10101,10 +10173,10 @@
         <v>922</v>
       </c>
       <c r="M156">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N156" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="157" spans="1:14">
@@ -10142,10 +10214,10 @@
         <v>922</v>
       </c>
       <c r="M157">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N157" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="158" spans="1:14">
@@ -10183,10 +10255,10 @@
         <v>922</v>
       </c>
       <c r="M158">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N158" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="159" spans="1:14">
@@ -10227,10 +10299,10 @@
         <v>920</v>
       </c>
       <c r="M159">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N159" t="s">
-        <v>1018</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="160" spans="1:14">
@@ -10268,10 +10340,10 @@
         <v>922</v>
       </c>
       <c r="M160">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N160" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="161" spans="1:14">
@@ -10312,10 +10384,10 @@
         <v>920</v>
       </c>
       <c r="M161">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N161" t="s">
-        <v>1018</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="162" spans="1:14">
@@ -10353,10 +10425,10 @@
         <v>922</v>
       </c>
       <c r="M162">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N162" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="163" spans="1:14">
@@ -10394,10 +10466,10 @@
         <v>922</v>
       </c>
       <c r="M163">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N163" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="164" spans="1:14">
@@ -10438,10 +10510,10 @@
         <v>920</v>
       </c>
       <c r="M164">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N164" t="s">
-        <v>1018</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="165" spans="1:14">
@@ -10482,10 +10554,10 @@
         <v>921</v>
       </c>
       <c r="M165">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N165" t="s">
-        <v>1022</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="166" spans="1:14">
@@ -10526,10 +10598,10 @@
         <v>922</v>
       </c>
       <c r="M166">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N166" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="167" spans="1:14">
@@ -10558,10 +10630,10 @@
         <v>917</v>
       </c>
       <c r="M167">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N167" t="s">
-        <v>1026</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="168" spans="1:14">
@@ -10590,10 +10662,10 @@
         <v>917</v>
       </c>
       <c r="M168">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N168" t="s">
-        <v>1026</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="169" spans="1:14">
@@ -10622,10 +10694,10 @@
         <v>917</v>
       </c>
       <c r="M169">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N169" t="s">
-        <v>1026</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="170" spans="1:14">
@@ -10666,10 +10738,10 @@
         <v>922</v>
       </c>
       <c r="M170">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N170" t="s">
-        <v>1017</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="171" spans="1:14">
@@ -10707,7 +10779,10 @@
         <v>927</v>
       </c>
       <c r="M171">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="N171" t="s">
+        <v>1037</v>
       </c>
     </row>
     <row r="172" spans="1:14">
@@ -10748,10 +10823,10 @@
         <v>921</v>
       </c>
       <c r="M172">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N172" t="s">
-        <v>1026</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="173" spans="1:14">
@@ -10792,10 +10867,10 @@
         <v>921</v>
       </c>
       <c r="M173">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N173" t="s">
-        <v>1026</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="174" spans="1:14">
@@ -10833,10 +10908,10 @@
         <v>922</v>
       </c>
       <c r="M174">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N174" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="175" spans="1:14">
@@ -10877,10 +10952,10 @@
         <v>921</v>
       </c>
       <c r="M175">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N175" t="s">
-        <v>1026</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="176" spans="1:14">
@@ -10918,10 +10993,10 @@
         <v>922</v>
       </c>
       <c r="M176">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N176" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="177" spans="1:14">
@@ -10959,10 +11034,10 @@
         <v>922</v>
       </c>
       <c r="M177">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N177" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="178" spans="1:14">
@@ -11000,10 +11075,10 @@
         <v>922</v>
       </c>
       <c r="M178">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N178" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="179" spans="1:14">
@@ -11047,7 +11122,7 @@
         <v>4</v>
       </c>
       <c r="N179" t="s">
-        <v>1027</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="180" spans="1:14">
@@ -11085,10 +11160,10 @@
         <v>922</v>
       </c>
       <c r="M180">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N180" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="181" spans="1:14">
@@ -11129,10 +11204,10 @@
         <v>921</v>
       </c>
       <c r="M181">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N181" t="s">
-        <v>1028</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="182" spans="1:14">
@@ -11170,10 +11245,10 @@
         <v>922</v>
       </c>
       <c r="M182">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N182" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="183" spans="1:14">
@@ -11214,10 +11289,10 @@
         <v>920</v>
       </c>
       <c r="M183">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N183" t="s">
-        <v>1029</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="184" spans="1:14">
@@ -11258,10 +11333,10 @@
         <v>921</v>
       </c>
       <c r="M184">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N184" t="s">
-        <v>1030</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="185" spans="1:14">
@@ -11299,10 +11374,10 @@
         <v>922</v>
       </c>
       <c r="M185">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N185" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="186" spans="1:14">
@@ -11340,10 +11415,10 @@
         <v>922</v>
       </c>
       <c r="M186">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N186" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="187" spans="1:14">
@@ -11381,10 +11456,10 @@
         <v>922</v>
       </c>
       <c r="M187">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N187" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="188" spans="1:14">
@@ -11422,10 +11497,10 @@
         <v>922</v>
       </c>
       <c r="M188">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N188" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="189" spans="1:14">
@@ -11460,10 +11535,10 @@
         <v>922</v>
       </c>
       <c r="M189">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N189" t="s">
-        <v>1015</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="190" spans="1:14">
@@ -11527,10 +11602,10 @@
         <v>922</v>
       </c>
       <c r="M191">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N191" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="192" spans="1:14">
@@ -11568,10 +11643,10 @@
         <v>931</v>
       </c>
       <c r="M192">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N192" t="s">
-        <v>1031</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="193" spans="1:14">
@@ -11606,10 +11681,10 @@
         <v>922</v>
       </c>
       <c r="M193">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N193" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="194" spans="1:14">
@@ -11647,10 +11722,10 @@
         <v>935</v>
       </c>
       <c r="M194">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N194" t="s">
-        <v>1029</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="195" spans="1:14">
@@ -11688,10 +11763,10 @@
         <v>949</v>
       </c>
       <c r="M195">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N195" t="s">
-        <v>1026</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="196" spans="1:14">
@@ -11729,10 +11804,10 @@
         <v>932</v>
       </c>
       <c r="M196">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N196" t="s">
-        <v>1029</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="197" spans="1:14">
@@ -11770,10 +11845,10 @@
         <v>932</v>
       </c>
       <c r="M197">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N197" t="s">
-        <v>1027</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="198" spans="1:14">
@@ -11811,10 +11886,10 @@
         <v>930</v>
       </c>
       <c r="M198">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N198" t="s">
-        <v>1026</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="199" spans="1:14">
@@ -11852,10 +11927,10 @@
         <v>934</v>
       </c>
       <c r="M199">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N199" t="s">
-        <v>1029</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="200" spans="1:14">
@@ -11890,10 +11965,10 @@
         <v>922</v>
       </c>
       <c r="M200">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N200" t="s">
-        <v>1032</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="201" spans="1:14">
@@ -11931,10 +12006,10 @@
         <v>941</v>
       </c>
       <c r="M201">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N201" t="s">
-        <v>1029</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="202" spans="1:14">
@@ -11972,10 +12047,10 @@
         <v>927</v>
       </c>
       <c r="M202">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N202" t="s">
-        <v>1026</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="203" spans="1:14">
@@ -12010,10 +12085,10 @@
         <v>922</v>
       </c>
       <c r="M203">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N203" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="204" spans="1:14">
@@ -12048,10 +12123,10 @@
         <v>922</v>
       </c>
       <c r="M204">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N204" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="205" spans="1:14">
@@ -12086,10 +12161,10 @@
         <v>922</v>
       </c>
       <c r="M205">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N205" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="206" spans="1:14">
@@ -12127,10 +12202,10 @@
         <v>933</v>
       </c>
       <c r="M206">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N206" t="s">
-        <v>1026</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="207" spans="1:14">
@@ -12165,10 +12240,10 @@
         <v>922</v>
       </c>
       <c r="M207">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N207" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="208" spans="1:14">
@@ -12203,10 +12278,10 @@
         <v>922</v>
       </c>
       <c r="M208">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N208" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="209" spans="1:14">
@@ -12244,10 +12319,10 @@
         <v>935</v>
       </c>
       <c r="M209">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N209" t="s">
-        <v>1029</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="210" spans="1:14">
@@ -12282,10 +12357,10 @@
         <v>922</v>
       </c>
       <c r="M210">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N210" t="s">
-        <v>1015</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="211" spans="1:14">
@@ -12323,10 +12398,10 @@
         <v>933</v>
       </c>
       <c r="M211">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N211" t="s">
-        <v>1033</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="212" spans="1:14">
@@ -12364,10 +12439,10 @@
         <v>922</v>
       </c>
       <c r="M212">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N212" t="s">
-        <v>1034</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="213" spans="1:14">
@@ -12405,10 +12480,10 @@
         <v>921</v>
       </c>
       <c r="M213">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N213" t="s">
-        <v>1035</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="214" spans="1:14">
@@ -12449,10 +12524,10 @@
         <v>921</v>
       </c>
       <c r="M214">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N214" t="s">
-        <v>1036</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="215" spans="1:14">
@@ -12493,10 +12568,10 @@
         <v>921</v>
       </c>
       <c r="M215">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N215" t="s">
-        <v>1037</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="216" spans="1:14">
@@ -12534,10 +12609,10 @@
         <v>922</v>
       </c>
       <c r="M216">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N216" t="s">
-        <v>1034</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="217" spans="1:14">
@@ -12575,10 +12650,10 @@
         <v>922</v>
       </c>
       <c r="M217">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N217" t="s">
-        <v>1034</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="218" spans="1:14">
@@ -12616,10 +12691,10 @@
         <v>922</v>
       </c>
       <c r="M218">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N218" t="s">
-        <v>1034</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="219" spans="1:14">
@@ -12657,10 +12732,10 @@
         <v>922</v>
       </c>
       <c r="M219">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N219" t="s">
-        <v>1034</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="220" spans="1:14">
@@ -12701,10 +12776,10 @@
         <v>920</v>
       </c>
       <c r="M220">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N220" t="s">
-        <v>1037</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="221" spans="1:14">
@@ -12783,10 +12858,10 @@
         <v>922</v>
       </c>
       <c r="M222">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N222" t="s">
-        <v>1034</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="223" spans="1:14">
@@ -12868,10 +12943,10 @@
         <v>921</v>
       </c>
       <c r="M224">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N224" t="s">
-        <v>1037</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="225" spans="1:14">
@@ -12909,10 +12984,10 @@
         <v>922</v>
       </c>
       <c r="M225">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N225" t="s">
-        <v>1034</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="226" spans="1:14">
@@ -12950,10 +13025,10 @@
         <v>922</v>
       </c>
       <c r="M226">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N226" t="s">
-        <v>1034</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="227" spans="1:14">
@@ -12991,10 +13066,10 @@
         <v>921</v>
       </c>
       <c r="M227">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N227" t="s">
-        <v>1035</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="228" spans="1:14">
@@ -13035,10 +13110,10 @@
         <v>920</v>
       </c>
       <c r="M228">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N228" t="s">
-        <v>1038</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="229" spans="1:14">
@@ -13079,10 +13154,10 @@
         <v>921</v>
       </c>
       <c r="M229">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N229" t="s">
-        <v>1037</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="230" spans="1:14">
@@ -13123,10 +13198,10 @@
         <v>922</v>
       </c>
       <c r="M230">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N230" t="s">
-        <v>1039</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="231" spans="1:14">
@@ -13167,10 +13242,10 @@
         <v>922</v>
       </c>
       <c r="M231">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N231" t="s">
-        <v>1039</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="232" spans="1:14">
@@ -13211,10 +13286,10 @@
         <v>922</v>
       </c>
       <c r="M232">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N232" t="s">
-        <v>1039</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="233" spans="1:14">
@@ -13255,10 +13330,10 @@
         <v>921</v>
       </c>
       <c r="M233">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N233" t="s">
-        <v>1039</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="234" spans="1:14">
@@ -13296,10 +13371,10 @@
         <v>920</v>
       </c>
       <c r="M234">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N234" t="s">
-        <v>1040</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="235" spans="1:14">
@@ -13340,10 +13415,10 @@
         <v>922</v>
       </c>
       <c r="M235">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N235" t="s">
-        <v>1039</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="236" spans="1:14">
@@ -13384,10 +13459,10 @@
         <v>920</v>
       </c>
       <c r="M236">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N236" t="s">
-        <v>1041</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="237" spans="1:14">
@@ -13428,10 +13503,10 @@
         <v>920</v>
       </c>
       <c r="M237">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N237" t="s">
-        <v>1039</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="238" spans="1:14">
@@ -13469,10 +13544,10 @@
         <v>922</v>
       </c>
       <c r="M238">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N238" t="s">
-        <v>1039</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="239" spans="1:14">
@@ -13513,10 +13588,10 @@
         <v>921</v>
       </c>
       <c r="M239">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N239" t="s">
-        <v>1039</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="240" spans="1:14">
@@ -13557,10 +13632,10 @@
         <v>922</v>
       </c>
       <c r="M240">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N240" t="s">
-        <v>1039</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="241" spans="1:14">
@@ -13598,10 +13673,10 @@
         <v>922</v>
       </c>
       <c r="M241">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N241" t="s">
-        <v>1039</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="242" spans="1:14">
@@ -13642,10 +13717,10 @@
         <v>920</v>
       </c>
       <c r="M242">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N242" t="s">
-        <v>1041</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="243" spans="1:14">
@@ -13686,10 +13761,10 @@
         <v>920</v>
       </c>
       <c r="M243">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N243" t="s">
-        <v>1041</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="244" spans="1:14">
@@ -13730,10 +13805,10 @@
         <v>922</v>
       </c>
       <c r="M244">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N244" t="s">
-        <v>1042</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="245" spans="1:14">
@@ -13774,10 +13849,10 @@
         <v>920</v>
       </c>
       <c r="M245">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N245" t="s">
-        <v>1043</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="246" spans="1:14">
@@ -13818,10 +13893,10 @@
         <v>920</v>
       </c>
       <c r="M246">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N246" t="s">
-        <v>1044</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="247" spans="1:14">
@@ -13862,10 +13937,10 @@
         <v>920</v>
       </c>
       <c r="M247">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N247" t="s">
-        <v>1044</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="248" spans="1:14">
@@ -13906,10 +13981,10 @@
         <v>922</v>
       </c>
       <c r="M248">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N248" t="s">
-        <v>1043</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="249" spans="1:14">
@@ -13950,10 +14025,10 @@
         <v>920</v>
       </c>
       <c r="M249">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N249" t="s">
-        <v>1044</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="250" spans="1:14">
@@ -13994,10 +14069,10 @@
         <v>922</v>
       </c>
       <c r="M250">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N250" t="s">
-        <v>1043</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="251" spans="1:14">
@@ -14038,10 +14113,10 @@
         <v>922</v>
       </c>
       <c r="M251">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N251" t="s">
-        <v>1043</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="252" spans="1:14">
@@ -14082,10 +14157,10 @@
         <v>920</v>
       </c>
       <c r="M252">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N252" t="s">
-        <v>1044</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="253" spans="1:14">
@@ -14126,10 +14201,10 @@
         <v>920</v>
       </c>
       <c r="M253">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N253" t="s">
-        <v>1044</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="254" spans="1:14">
@@ -14167,10 +14242,10 @@
         <v>922</v>
       </c>
       <c r="M254">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N254" t="s">
-        <v>1043</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="255" spans="1:14">
@@ -14211,10 +14286,10 @@
         <v>921</v>
       </c>
       <c r="M255">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N255" t="s">
-        <v>1045</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="256" spans="1:14">
@@ -14290,10 +14365,10 @@
         <v>921</v>
       </c>
       <c r="M257">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N257" t="s">
-        <v>1043</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="258" spans="1:14">
@@ -14334,10 +14409,10 @@
         <v>920</v>
       </c>
       <c r="M258">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N258" t="s">
-        <v>1044</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="259" spans="1:14">
@@ -14378,10 +14453,10 @@
         <v>921</v>
       </c>
       <c r="M259">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N259" t="s">
-        <v>1045</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="260" spans="1:14">
@@ -14419,10 +14494,10 @@
         <v>922</v>
       </c>
       <c r="M260">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N260" t="s">
-        <v>1043</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="261" spans="1:14">
@@ -14463,10 +14538,10 @@
         <v>920</v>
       </c>
       <c r="M261">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N261" t="s">
-        <v>1044</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="262" spans="1:14">
@@ -14504,10 +14579,10 @@
         <v>922</v>
       </c>
       <c r="M262">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N262" t="s">
-        <v>1043</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="263" spans="1:14">
@@ -14548,10 +14623,10 @@
         <v>920</v>
       </c>
       <c r="M263">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N263" t="s">
-        <v>1044</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="264" spans="1:14">
@@ -14592,10 +14667,10 @@
         <v>920</v>
       </c>
       <c r="M264">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N264" t="s">
-        <v>1044</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="265" spans="1:14">
@@ -14636,7 +14711,10 @@
         <v>922</v>
       </c>
       <c r="M265">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="N265" t="s">
+        <v>1068</v>
       </c>
     </row>
     <row r="266" spans="1:14">
@@ -14674,7 +14752,10 @@
         <v>922</v>
       </c>
       <c r="M266">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="N266" t="s">
+        <v>1068</v>
       </c>
     </row>
     <row r="267" spans="1:14">
@@ -14712,7 +14793,10 @@
         <v>922</v>
       </c>
       <c r="M267">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="N267" t="s">
+        <v>1068</v>
       </c>
     </row>
     <row r="268" spans="1:14">
@@ -14750,7 +14834,10 @@
         <v>922</v>
       </c>
       <c r="M268">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="N268" t="s">
+        <v>1068</v>
       </c>
     </row>
     <row r="269" spans="1:14">
@@ -14788,7 +14875,10 @@
         <v>922</v>
       </c>
       <c r="M269">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="N269" t="s">
+        <v>1068</v>
       </c>
     </row>
     <row r="270" spans="1:14">
@@ -14826,7 +14916,10 @@
         <v>922</v>
       </c>
       <c r="M270">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="N270" t="s">
+        <v>1037</v>
       </c>
     </row>
     <row r="271" spans="1:14">
@@ -14867,7 +14960,10 @@
         <v>920</v>
       </c>
       <c r="M271">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="N271" t="s">
+        <v>1069</v>
       </c>
     </row>
     <row r="272" spans="1:14">
@@ -14905,10 +15001,13 @@
         <v>922</v>
       </c>
       <c r="M272">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="273" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N272" t="s">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="273" spans="1:14">
       <c r="A273" t="s">
         <v>286</v>
       </c>
@@ -14946,10 +15045,13 @@
         <v>920</v>
       </c>
       <c r="M273">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="274" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N273" t="s">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="274" spans="1:14">
       <c r="A274" t="s">
         <v>287</v>
       </c>
@@ -14987,10 +15089,13 @@
         <v>922</v>
       </c>
       <c r="M274">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="275" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N274" t="s">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="275" spans="1:14">
       <c r="A275" t="s">
         <v>288</v>
       </c>
@@ -15028,10 +15133,13 @@
         <v>920</v>
       </c>
       <c r="M275">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="276" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N275" t="s">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="276" spans="1:14">
       <c r="A276" t="s">
         <v>289</v>
       </c>
@@ -15069,10 +15177,13 @@
         <v>922</v>
       </c>
       <c r="M276">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="277" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N276" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="277" spans="1:14">
       <c r="A277" t="s">
         <v>290</v>
       </c>
@@ -15110,10 +15221,13 @@
         <v>922</v>
       </c>
       <c r="M277">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="278" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N277" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="278" spans="1:14">
       <c r="A278" t="s">
         <v>291</v>
       </c>
@@ -15148,10 +15262,13 @@
         <v>922</v>
       </c>
       <c r="M278">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="279" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N278" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="279" spans="1:14">
       <c r="A279" t="s">
         <v>292</v>
       </c>
@@ -15189,10 +15306,13 @@
         <v>922</v>
       </c>
       <c r="M279">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="280" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N279" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="280" spans="1:14">
       <c r="A280" t="s">
         <v>293</v>
       </c>
@@ -15230,10 +15350,13 @@
         <v>922</v>
       </c>
       <c r="M280">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="281" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N280" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="281" spans="1:14">
       <c r="A281" t="s">
         <v>294</v>
       </c>
@@ -15271,10 +15394,13 @@
         <v>922</v>
       </c>
       <c r="M281">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="282" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N281" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="282" spans="1:14">
       <c r="A282" t="s">
         <v>295</v>
       </c>
@@ -15315,7 +15441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:13">
+    <row r="283" spans="1:14">
       <c r="A283" t="s">
         <v>296</v>
       </c>
@@ -15350,10 +15476,13 @@
         <v>922</v>
       </c>
       <c r="M283">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="284" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N283" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="284" spans="1:14">
       <c r="A284" t="s">
         <v>297</v>
       </c>
@@ -15388,10 +15517,13 @@
         <v>922</v>
       </c>
       <c r="M284">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="285" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N284" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="285" spans="1:14">
       <c r="A285" t="s">
         <v>298</v>
       </c>
@@ -15426,10 +15558,13 @@
         <v>922</v>
       </c>
       <c r="M285">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="286" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N285" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="286" spans="1:14">
       <c r="A286" t="s">
         <v>299</v>
       </c>
@@ -15464,10 +15599,13 @@
         <v>922</v>
       </c>
       <c r="M286">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="287" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N286" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="287" spans="1:14">
       <c r="A287" t="s">
         <v>300</v>
       </c>
@@ -15505,10 +15643,13 @@
         <v>920</v>
       </c>
       <c r="M287">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="288" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N287" t="s">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="288" spans="1:14">
       <c r="A288" t="s">
         <v>301</v>
       </c>
@@ -15543,10 +15684,13 @@
         <v>922</v>
       </c>
       <c r="M288">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="289" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N288" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="289" spans="1:14">
       <c r="A289" t="s">
         <v>302</v>
       </c>
@@ -15584,7 +15728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:13">
+    <row r="290" spans="1:14">
       <c r="A290" t="s">
         <v>303</v>
       </c>
@@ -15622,10 +15766,13 @@
         <v>922</v>
       </c>
       <c r="M290">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="291" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N290" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="291" spans="1:14">
       <c r="A291" t="s">
         <v>304</v>
       </c>
@@ -15663,10 +15810,13 @@
         <v>920</v>
       </c>
       <c r="M291">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="292" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N291" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="292" spans="1:14">
       <c r="A292" t="s">
         <v>305</v>
       </c>
@@ -15701,10 +15851,13 @@
         <v>922</v>
       </c>
       <c r="M292">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="293" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N292" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="293" spans="1:14">
       <c r="A293" t="s">
         <v>306</v>
       </c>
@@ -15739,10 +15892,13 @@
         <v>922</v>
       </c>
       <c r="M293">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="294" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N293" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="294" spans="1:14">
       <c r="A294" t="s">
         <v>307</v>
       </c>
@@ -15777,10 +15933,13 @@
         <v>922</v>
       </c>
       <c r="M294">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="295" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N294" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="295" spans="1:14">
       <c r="A295" t="s">
         <v>308</v>
       </c>
@@ -15818,10 +15977,13 @@
         <v>922</v>
       </c>
       <c r="M295">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="296" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N295" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="296" spans="1:14">
       <c r="A296" t="s">
         <v>309</v>
       </c>
@@ -15856,10 +16018,13 @@
         <v>922</v>
       </c>
       <c r="M296">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="297" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N296" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="297" spans="1:14">
       <c r="A297" t="s">
         <v>310</v>
       </c>
@@ -15894,10 +16059,13 @@
         <v>922</v>
       </c>
       <c r="M297">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="298" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N297" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="298" spans="1:14">
       <c r="A298" t="s">
         <v>311</v>
       </c>
@@ -15932,10 +16100,13 @@
         <v>922</v>
       </c>
       <c r="M298">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="299" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N298" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="299" spans="1:14">
       <c r="A299" t="s">
         <v>312</v>
       </c>
@@ -15976,7 +16147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:13">
+    <row r="300" spans="1:14">
       <c r="A300" t="s">
         <v>313</v>
       </c>
@@ -16014,10 +16185,13 @@
         <v>922</v>
       </c>
       <c r="M300">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="301" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N300" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="301" spans="1:14">
       <c r="A301" t="s">
         <v>314</v>
       </c>
@@ -16055,10 +16229,13 @@
         <v>922</v>
       </c>
       <c r="M301">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="302" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N301" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="302" spans="1:14">
       <c r="A302" t="s">
         <v>315</v>
       </c>
@@ -16093,10 +16270,13 @@
         <v>935</v>
       </c>
       <c r="M302">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="303" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N302" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="303" spans="1:14">
       <c r="A303" t="s">
         <v>316</v>
       </c>
@@ -16128,10 +16308,13 @@
         <v>922</v>
       </c>
       <c r="M303">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="304" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N303" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="304" spans="1:14">
       <c r="A304" t="s">
         <v>317</v>
       </c>
@@ -16163,10 +16346,13 @@
         <v>922</v>
       </c>
       <c r="M304">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="305" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N304" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="305" spans="1:14">
       <c r="A305" t="s">
         <v>318</v>
       </c>
@@ -16198,10 +16384,13 @@
         <v>922</v>
       </c>
       <c r="M305">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="306" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N305" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="306" spans="1:14">
       <c r="A306" t="s">
         <v>319</v>
       </c>
@@ -16236,10 +16425,13 @@
         <v>935</v>
       </c>
       <c r="M306">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="307" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N306" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="307" spans="1:14">
       <c r="A307" t="s">
         <v>320</v>
       </c>
@@ -16271,10 +16463,13 @@
         <v>922</v>
       </c>
       <c r="M307">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="308" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N307" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="308" spans="1:14">
       <c r="A308" t="s">
         <v>321</v>
       </c>
@@ -16306,10 +16501,13 @@
         <v>922</v>
       </c>
       <c r="M308">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="309" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N308" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="309" spans="1:14">
       <c r="A309" t="s">
         <v>322</v>
       </c>
@@ -16341,10 +16539,13 @@
         <v>922</v>
       </c>
       <c r="M309">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="310" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N309" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="310" spans="1:14">
       <c r="A310" t="s">
         <v>323</v>
       </c>
@@ -16382,7 +16583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:13">
+    <row r="311" spans="1:14">
       <c r="A311" t="s">
         <v>324</v>
       </c>
@@ -16417,10 +16618,13 @@
         <v>970</v>
       </c>
       <c r="M311">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="312" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N311" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="312" spans="1:14">
       <c r="A312" t="s">
         <v>325</v>
       </c>
@@ -16455,10 +16659,13 @@
         <v>932</v>
       </c>
       <c r="M312">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="313" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N312" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="313" spans="1:14">
       <c r="A313" t="s">
         <v>326</v>
       </c>
@@ -16493,10 +16700,13 @@
         <v>930</v>
       </c>
       <c r="M313">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="314" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="N313" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="314" spans="1:14">
       <c r="A314" t="s">
         <v>327</v>
       </c>
@@ -16531,7 +16741,10 @@
         <v>933</v>
       </c>
       <c r="M314">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="N314" t="s">
+        <v>1068</v>
       </c>
     </row>
   </sheetData>

</xml_diff>